<commit_message>
[feat] New file template
</commit_message>
<xml_diff>
--- a/public/Files/codeTemplate.xlsx
+++ b/public/Files/codeTemplate.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aleena Chaudhry\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Moamen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E1A9C1-1322-41FE-B3C2-6628CD3D0E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CN2022" sheetId="1" r:id="rId1"/>
@@ -28,13 +29,13 @@
     <t>Code</t>
   </si>
   <si>
-    <t>Monetary Values</t>
+    <t>Valeur totale en €</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -84,7 +85,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -159,6 +160,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -194,6 +212,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -369,11 +404,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" customWidth="1"/>
+    <col min="1" max="1" width="19.90625" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>